<commit_message>
Cerrar comparador de validacion y tabla descriptiva; armonizar materiales
</commit_message>
<xml_diff>
--- a/results/tables/STROBE_checklist.xlsx
+++ b/results/tables/STROBE_checklist.xlsx
@@ -702,7 +702,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra y Figura 1 (exclusión de presión arterial no válida, embarazo y ponderador faltante, cada una con su n); Materiales y métodos &gt; Modelo estadístico (seis registros de control de dos municipios sin pobreza publicada por CONEVAL 2020; Tabla S1). Los datos faltantes por covariable no se tabulan en el manuscrito</t>
+          <t>Resultados &gt; Muestra y Figura 1 (exclusión de presión arterial no válida, embarazo y ponderador faltante, cada una con su n); Materiales y métodos &gt; Modelo estadístico (seis registros de control de dos municipios sin pobreza publicada por CONEVAL 2020; Tabla S1). Tabla S8, panel B (faltantes por covariable y denominador)</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra; Cuadro I (n por año). Las características sociodemográficas de los participantes no se tabulan en el manuscrito</t>
+          <t>Resultados &gt; Muestra; Cuadro I (n por año). Tabla S8, panel A (características por denominador)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Resultados &gt; Muestra; Figura 1 (flujo con el n de cada exclusión); Cuadro I; Materiales y métodos &gt; Modelo estadístico (registros sin pobreza municipal)</t>
+          <t>Resultados &gt; Muestra; Figura 1 (flujo con el n de cada exclusión); Cuadro I; Materiales y métodos &gt; Modelo estadístico (registros sin pobreza municipal); Tabla S8, panel B</t>
         </is>
       </c>
     </row>

</xml_diff>